<commit_message>
fix(web): no-issue: register React Testing Library cleanup explicitly
RTL only registers its own `afterEach(cleanup)` when a global `afterEach` exists, which is to
say when `globals: true` is set. Dropping that flag (this suite imports its test functions
explicitly, so a missing import is a lint error rather than a runtime one) left each test
rendering into the DOM the previous one had left behind, failing 46 cases on `getBy*` queries
that matched more than one element. Register the cleanup in a setup file instead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/central-server/exported-refdata-all-table.xlsx
+++ b/packages/central-server/exported-refdata-all-table.xlsx
@@ -445,22 +445,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>621730af-3caa-46a9-bea4-516276cb74e2</v>
+        <v>e09e9910-d3e0-42cf-8477-1574b4354279</v>
       </c>
       <c r="B2" t="str">
-        <v>CZTT072107</v>
+        <v>VWTJ063395</v>
       </c>
       <c r="C2" t="str">
-        <v>Agnes</v>
+        <v>Lelia</v>
       </c>
       <c r="E2" t="str">
-        <v>Marinai</v>
+        <v>Allen</v>
       </c>
       <c r="F2" t="str">
-        <v>Bertin</v>
+        <v>Kirby</v>
       </c>
       <c r="G2" s="1">
-        <v>25456</v>
+        <v>27474</v>
       </c>
       <c r="I2" t="str">
         <v>female</v>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -493,6 +493,9 @@
       <c r="D1" t="str">
         <v>visibilityStatus</v>
       </c>
+      <c r="E1" t="str">
+        <v>availableFacilities</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -524,14 +527,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -546,6 +549,9 @@
       <c r="D1" t="str">
         <v>visibilityStatus</v>
       </c>
+      <c r="E1" t="str">
+        <v>availableFacilities</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -577,7 +583,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
read drug facility columns from header
</commit_message>
<xml_diff>
--- a/packages/central-server/exported-refdata-all-table.xlsx
+++ b/packages/central-server/exported-refdata-all-table.xlsx
@@ -445,25 +445,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>e09e9910-d3e0-42cf-8477-1574b4354279</v>
+        <v>1ed6a4ae-ca3a-4aba-8c8f-01a4e632f3c4</v>
       </c>
       <c r="B2" t="str">
-        <v>VWTJ063395</v>
+        <v>OSUC515697</v>
       </c>
       <c r="C2" t="str">
-        <v>Lelia</v>
+        <v>David</v>
       </c>
       <c r="E2" t="str">
-        <v>Allen</v>
+        <v>Bucelli</v>
       </c>
       <c r="F2" t="str">
-        <v>Kirby</v>
+        <v>Bos</v>
       </c>
       <c r="G2" s="1">
-        <v>27474</v>
+        <v>29915</v>
       </c>
       <c r="I2" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="K2" t="str">
         <v>current</v>

</xml_diff>

<commit_message>
fix(medications): no-issue: allow a drug reference data export to be re-imported (HOTFIX 2.64) (#10995)
read drug facility columns from header
</commit_message>
<xml_diff>
--- a/packages/central-server/exported-refdata-all-table.xlsx
+++ b/packages/central-server/exported-refdata-all-table.xlsx
@@ -445,25 +445,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>e09e9910-d3e0-42cf-8477-1574b4354279</v>
+        <v>1ed6a4ae-ca3a-4aba-8c8f-01a4e632f3c4</v>
       </c>
       <c r="B2" t="str">
-        <v>VWTJ063395</v>
+        <v>OSUC515697</v>
       </c>
       <c r="C2" t="str">
-        <v>Lelia</v>
+        <v>David</v>
       </c>
       <c r="E2" t="str">
-        <v>Allen</v>
+        <v>Bucelli</v>
       </c>
       <c r="F2" t="str">
-        <v>Kirby</v>
+        <v>Bos</v>
       </c>
       <c r="G2" s="1">
-        <v>27474</v>
+        <v>29915</v>
       </c>
       <c r="I2" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="K2" t="str">
         <v>current</v>

</xml_diff>